<commit_message>
Fill final gate-fix result (Llama arm): manuscript 5.7, blue copy, response letter R1.2 — all placeholders resolved
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/llama3_2_latest__gatefix/comparison_SelfCorrectionRAG/SelfCorrectionRAG_costs.xlsx
+++ b/results/llama3_2_latest__gatefix/comparison_SelfCorrectionRAG/SelfCorrectionRAG_costs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -472,13 +472,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7.416308641433716</v>
+        <v>98.44901013374329</v>
       </c>
       <c r="B2" t="n">
-        <v>1502.359375</v>
+        <v>196.09375</v>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>6.2</v>
       </c>
       <c r="D2" t="n">
         <v>4</v>
@@ -487,10 +487,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>1.075171232223511</v>
+        <v>1.974961996078491</v>
       </c>
       <c r="G2" t="n">
-        <v>1.078155040740967</v>
+        <v>37.80867099761963</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -498,13 +498,13 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.04212021827698</v>
+        <v>80.98165202140808</v>
       </c>
       <c r="B3" t="n">
-        <v>1502.90234375</v>
+        <v>139.234375</v>
       </c>
       <c r="C3" t="n">
-        <v>10.1</v>
+        <v>6.9</v>
       </c>
       <c r="D3" t="n">
         <v>4</v>
@@ -513,10 +513,10 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1.5174560546875</v>
+        <v>2.944238185882568</v>
       </c>
       <c r="G3" t="n">
-        <v>1.519016027450562</v>
+        <v>29.74052214622498</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -524,13 +524,13 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>11.06787991523743</v>
+        <v>80.6724648475647</v>
       </c>
       <c r="B4" t="n">
-        <v>1503.2890625</v>
+        <v>143.75</v>
       </c>
       <c r="C4" t="n">
-        <v>10.2</v>
+        <v>6.1</v>
       </c>
       <c r="D4" t="n">
         <v>4</v>
@@ -539,10 +539,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>1.499449968338013</v>
+        <v>2.559149026870728</v>
       </c>
       <c r="G4" t="n">
-        <v>1.501154899597168</v>
+        <v>40.09256076812744</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -550,25 +550,25 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>11.57150030136108</v>
+        <v>32.07939291000366</v>
       </c>
       <c r="B5" t="n">
-        <v>1503.33984375</v>
+        <v>144.421875</v>
       </c>
       <c r="C5" t="n">
-        <v>9.4</v>
+        <v>3.7</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>2.538486480712891</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>2.54012393951416</v>
+        <v>32.07938885688782</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -576,25 +576,25 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>11.0548632144928</v>
+        <v>36.28087973594666</v>
       </c>
       <c r="B6" t="n">
-        <v>1503.58203125</v>
+        <v>143.171875</v>
       </c>
       <c r="C6" t="n">
-        <v>7.8</v>
+        <v>5.6</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>2.51356315612793</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>2.515053033828735</v>
+        <v>36.28086876869202</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -602,25 +602,25 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>13.68193173408508</v>
+        <v>1985.307137012482</v>
       </c>
       <c r="B7" t="n">
-        <v>1504.91796875</v>
+        <v>37.265625</v>
       </c>
       <c r="C7" t="n">
-        <v>10.4</v>
+        <v>6.8</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>1.481336832046509</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1.48303484916687</v>
+        <v>1985.307085037231</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -628,25 +628,25 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10.56893277168274</v>
+        <v>102.6565487384796</v>
       </c>
       <c r="B8" t="n">
-        <v>1504.91796875</v>
+        <v>32.484375</v>
       </c>
       <c r="C8" t="n">
-        <v>8.9</v>
+        <v>4.4</v>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>1.484270572662354</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>1.48605489730835</v>
+        <v>102.6565148830414</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -654,13 +654,13 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>4.290479421615601</v>
+        <v>175.2775340080261</v>
       </c>
       <c r="B9" t="n">
-        <v>1504.91796875</v>
+        <v>106.609375</v>
       </c>
       <c r="C9" t="n">
-        <v>12.5</v>
+        <v>6.3</v>
       </c>
       <c r="D9" t="n">
         <v>4</v>
@@ -669,10 +669,10 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>1.485265493392944</v>
+        <v>4.023576974868774</v>
       </c>
       <c r="G9" t="n">
-        <v>1.486840009689331</v>
+        <v>105.5454730987549</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -680,13 +680,13 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2.373820304870605</v>
+        <v>155.859249830246</v>
       </c>
       <c r="B10" t="n">
-        <v>1504.91796875</v>
+        <v>41.890625</v>
       </c>
       <c r="C10" t="n">
-        <v>7.3</v>
+        <v>3.6</v>
       </c>
       <c r="D10" t="n">
         <v>4</v>
@@ -695,10 +695,10 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0.4668910503387451</v>
+        <v>2.421268939971924</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4685661792755127</v>
+        <v>77.42440891265869</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -706,13 +706,13 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>12.0915265083313</v>
+        <v>130.7491688728333</v>
       </c>
       <c r="B11" t="n">
-        <v>1504.91796875</v>
+        <v>38.03125</v>
       </c>
       <c r="C11" t="n">
-        <v>10.9</v>
+        <v>7.2</v>
       </c>
       <c r="D11" t="n">
         <v>4</v>
@@ -721,10 +721,10 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.399059534072876</v>
+        <v>3.031794309616089</v>
       </c>
       <c r="G11" t="n">
-        <v>0.4006154537200928</v>
+        <v>63.4993622303009</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -732,25 +732,25 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10.56877565383911</v>
+        <v>93.94772005081177</v>
       </c>
       <c r="B12" t="n">
-        <v>1504.921875</v>
+        <v>26.484375</v>
       </c>
       <c r="C12" t="n">
-        <v>9.6</v>
+        <v>11.2</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>1.455920219421387</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>1.457530975341797</v>
+        <v>93.94767928123474</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -758,13 +758,13 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11.13385796546936</v>
+        <v>156.8315689563751</v>
       </c>
       <c r="B13" t="n">
-        <v>1505.24609375</v>
+        <v>39.625</v>
       </c>
       <c r="C13" t="n">
-        <v>8.699999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="D13" t="n">
         <v>4</v>
@@ -773,10 +773,10 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>1.483949184417725</v>
+        <v>3.926463842391968</v>
       </c>
       <c r="G13" t="n">
-        <v>1.485470056533813</v>
+        <v>85.08348488807678</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -784,13 +784,13 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>10.40467143058777</v>
+        <v>139.3563277721405</v>
       </c>
       <c r="B14" t="n">
-        <v>1505.5625</v>
+        <v>39.46875</v>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>4.9</v>
       </c>
       <c r="D14" t="n">
         <v>4</v>
@@ -799,10 +799,10 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>1.564459562301636</v>
+        <v>2.741819143295288</v>
       </c>
       <c r="G14" t="n">
-        <v>1.566574096679688</v>
+        <v>66.50416898727417</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -810,13 +810,13 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4.041972637176514</v>
+        <v>113.7983701229095</v>
       </c>
       <c r="B15" t="n">
-        <v>1505.5625</v>
+        <v>85.421875</v>
       </c>
       <c r="C15" t="n">
-        <v>7.2</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
         <v>4</v>
@@ -825,10 +825,10 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>2.564634799957275</v>
+        <v>2.529568910598755</v>
       </c>
       <c r="G15" t="n">
-        <v>2.566180944442749</v>
+        <v>54.16732096672058</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -836,25 +836,25 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2.722403526306152</v>
+        <v>105.8721721172333</v>
       </c>
       <c r="B16" t="n">
-        <v>1505.56640625</v>
+        <v>36.25</v>
       </c>
       <c r="C16" t="n">
-        <v>9.6</v>
+        <v>4.2</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>1.453002691268921</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>1.454621553421021</v>
+        <v>105.8721449375153</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -862,13 +862,13 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1.138053894042969</v>
+        <v>149.7484121322632</v>
       </c>
       <c r="B17" t="n">
-        <v>1506.00390625</v>
+        <v>23.03125</v>
       </c>
       <c r="C17" t="n">
-        <v>6.4</v>
+        <v>11</v>
       </c>
       <c r="D17" t="n">
         <v>4</v>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.3933370113372803</v>
+        <v>3.591459989547729</v>
       </c>
       <c r="G17" t="n">
-        <v>0.3949875831604004</v>
+        <v>93.34073901176453</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -888,25 +888,25 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>14.07056045532227</v>
+        <v>87.2583441734314</v>
       </c>
       <c r="B18" t="n">
-        <v>1506.00390625</v>
+        <v>26.4375</v>
       </c>
       <c r="C18" t="n">
-        <v>10</v>
+        <v>11.5</v>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>1.45282769203186</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>1.454415559768677</v>
+        <v>87.25832319259644</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -914,25 +914,25 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>9.735885143280029</v>
+        <v>125.6786150932312</v>
       </c>
       <c r="B19" t="n">
-        <v>1506.00390625</v>
+        <v>24.109375</v>
       </c>
       <c r="C19" t="n">
-        <v>10.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>1.493953704833984</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>1.495516777038574</v>
+        <v>125.6785950660706</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -940,25 +940,25 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>11.53684520721436</v>
+        <v>61.35710883140564</v>
       </c>
       <c r="B20" t="n">
-        <v>1506.23828125</v>
+        <v>24.15625</v>
       </c>
       <c r="C20" t="n">
-        <v>8.9</v>
+        <v>5.6</v>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>1.498727798461914</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>1.500492572784424</v>
+        <v>61.35707783699036</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -966,13 +966,13 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>13.09890460968018</v>
+        <v>2538.310411214828</v>
       </c>
       <c r="B21" t="n">
-        <v>1509.13671875</v>
+        <v>50.5625</v>
       </c>
       <c r="C21" t="n">
-        <v>9.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D21" t="n">
         <v>4</v>
@@ -981,10 +981,10 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>1.710393190383911</v>
+        <v>3.422324895858765</v>
       </c>
       <c r="G21" t="n">
-        <v>1.712727069854736</v>
+        <v>2359.284959077835</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -992,13 +992,13 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>10.24337339401245</v>
+        <v>342.8620727062225</v>
       </c>
       <c r="B22" t="n">
-        <v>1509.13671875</v>
+        <v>39.4375</v>
       </c>
       <c r="C22" t="n">
-        <v>9.300000000000001</v>
+        <v>4.1</v>
       </c>
       <c r="D22" t="n">
         <v>4</v>
@@ -1007,10 +1007,10 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>1.445538997650146</v>
+        <v>2.591594934463501</v>
       </c>
       <c r="G22" t="n">
-        <v>1.447184562683105</v>
+        <v>150.192587852478</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1018,13 +1018,13 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>10.06352853775024</v>
+        <v>181.7903079986572</v>
       </c>
       <c r="B23" t="n">
-        <v>1509.13671875</v>
+        <v>38.328125</v>
       </c>
       <c r="C23" t="n">
-        <v>10.4</v>
+        <v>3.8</v>
       </c>
       <c r="D23" t="n">
         <v>4</v>
@@ -1033,10 +1033,10 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>1.51862096786499</v>
+        <v>3.106200695037842</v>
       </c>
       <c r="G23" t="n">
-        <v>1.52019739151001</v>
+        <v>110.0732898712158</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1044,25 +1044,25 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>10.42429184913635</v>
+        <v>31.87324810028076</v>
       </c>
       <c r="B24" t="n">
-        <v>1509.13671875</v>
+        <v>47.546875</v>
       </c>
       <c r="C24" t="n">
-        <v>10.4</v>
+        <v>4.3</v>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>1.447219848632812</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>1.448699235916138</v>
+        <v>31.8732430934906</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1070,25 +1070,25 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3.062867879867554</v>
+        <v>29.39018201828003</v>
       </c>
       <c r="B25" t="n">
-        <v>1509.13671875</v>
+        <v>48</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>3.1</v>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.54695725440979</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>2.548557281494141</v>
+        <v>29.3901789188385</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1096,25 +1096,25 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2.11370062828064</v>
+        <v>30.50363492965698</v>
       </c>
       <c r="B26" t="n">
-        <v>1509.13671875</v>
+        <v>48.234375</v>
       </c>
       <c r="C26" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="D26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>1.361691474914551</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>1.363716602325439</v>
+        <v>30.5036301612854</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1122,25 +1122,25 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3.139597177505493</v>
+        <v>26.62699007987976</v>
       </c>
       <c r="B27" t="n">
-        <v>1509.13671875</v>
+        <v>48.375</v>
       </c>
       <c r="C27" t="n">
-        <v>8</v>
+        <v>3.7</v>
       </c>
       <c r="D27" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>1.386247634887695</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>1.388109683990479</v>
+        <v>26.62698698043823</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1148,25 +1148,25 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2.272003173828125</v>
+        <v>29.33649182319641</v>
       </c>
       <c r="B28" t="n">
-        <v>1509.13671875</v>
+        <v>49.6875</v>
       </c>
       <c r="C28" t="n">
-        <v>12.9</v>
+        <v>3.5</v>
       </c>
       <c r="D28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>1.368595600128174</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>1.370246648788452</v>
+        <v>29.33648705482483</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -1174,25 +1174,25 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1.895581007003784</v>
+        <v>30.93264412879944</v>
       </c>
       <c r="B29" t="n">
-        <v>1509.13671875</v>
+        <v>49.46875</v>
       </c>
       <c r="C29" t="n">
-        <v>3.1</v>
+        <v>14.1</v>
       </c>
       <c r="D29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>1.397442579269409</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>1.39905834197998</v>
+        <v>30.93264102935791</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -1200,13 +1200,13 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>11.87508130073547</v>
+        <v>93.63500499725342</v>
       </c>
       <c r="B30" t="n">
-        <v>1509.13671875</v>
+        <v>83.15625</v>
       </c>
       <c r="C30" t="n">
-        <v>10.4</v>
+        <v>4.2</v>
       </c>
       <c r="D30" t="n">
         <v>4</v>
@@ -1215,10 +1215,10 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>1.419911623001099</v>
+        <v>3.022176027297974</v>
       </c>
       <c r="G30" t="n">
-        <v>1.421907186508179</v>
+        <v>45.48308300971985</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -1226,13 +1226,13 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3.4451584815979</v>
+        <v>105.1430802345276</v>
       </c>
       <c r="B31" t="n">
-        <v>1509.13671875</v>
+        <v>89.9375</v>
       </c>
       <c r="C31" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
         <v>4</v>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>2.559489488601685</v>
+        <v>2.659034967422485</v>
       </c>
       <c r="G31" t="n">
-        <v>2.5610191822052</v>
+        <v>52.74488711357117</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -1252,25 +1252,25 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1.575536727905273</v>
+        <v>52.87909507751465</v>
       </c>
       <c r="B32" t="n">
-        <v>1509.13671875</v>
+        <v>90.359375</v>
       </c>
       <c r="C32" t="n">
-        <v>7.3</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0.3248918056488037</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0.3264880180358887</v>
+        <v>52.87908887863159</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1278,25 +1278,25 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>10.21217250823975</v>
+        <v>73.89662909507751</v>
       </c>
       <c r="B33" t="n">
-        <v>1509.13671875</v>
+        <v>89.65625</v>
       </c>
       <c r="C33" t="n">
-        <v>11.5</v>
+        <v>3.1</v>
       </c>
       <c r="D33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>0.3448114395141602</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0.3465657234191895</v>
+        <v>73.8966269493103</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -1304,25 +1304,25 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>13.8501513004303</v>
+        <v>41.59338092803955</v>
       </c>
       <c r="B34" t="n">
-        <v>1509.13671875</v>
+        <v>37.1875</v>
       </c>
       <c r="C34" t="n">
-        <v>10.1</v>
+        <v>14.7</v>
       </c>
       <c r="D34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>1.452259540557861</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>1.453809261322021</v>
+        <v>41.59333992004395</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -1330,13 +1330,13 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>11.57649636268616</v>
+        <v>140.1787841320038</v>
       </c>
       <c r="B35" t="n">
-        <v>1509.13671875</v>
+        <v>38.421875</v>
       </c>
       <c r="C35" t="n">
-        <v>10.5</v>
+        <v>6.5</v>
       </c>
       <c r="D35" t="n">
         <v>4</v>
@@ -1345,10 +1345,10 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>1.21482253074646</v>
+        <v>2.880224943161011</v>
       </c>
       <c r="G35" t="n">
-        <v>1.216347694396973</v>
+        <v>70.03197503089905</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1356,13 +1356,13 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>9.967308044433594</v>
+        <v>117.9811089038849</v>
       </c>
       <c r="B36" t="n">
-        <v>1509.140625</v>
+        <v>85.140625</v>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>3.6</v>
       </c>
       <c r="D36" t="n">
         <v>4</v>
@@ -1371,10 +1371,10 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>1.460657119750977</v>
+        <v>3.463802814483643</v>
       </c>
       <c r="G36" t="n">
-        <v>1.462340354919434</v>
+        <v>52.61568570137024</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -1382,13 +1382,13 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3.299293518066406</v>
+        <v>136.8003759384155</v>
       </c>
       <c r="B37" t="n">
-        <v>1509.24609375</v>
+        <v>88.25</v>
       </c>
       <c r="C37" t="n">
-        <v>9.6</v>
+        <v>3.3</v>
       </c>
       <c r="D37" t="n">
         <v>4</v>
@@ -1397,10 +1397,10 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>1.457995653152466</v>
+        <v>2.602930784225464</v>
       </c>
       <c r="G37" t="n">
-        <v>1.459661722183228</v>
+        <v>50.02520799636841</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -1408,25 +1408,25 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1.042274236679077</v>
+        <v>73.05420994758606</v>
       </c>
       <c r="B38" t="n">
-        <v>1509.359375</v>
+        <v>37.625</v>
       </c>
       <c r="C38" t="n">
-        <v>6.8</v>
+        <v>3.3</v>
       </c>
       <c r="D38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0.3469047546386719</v>
+        <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0.3484566211700439</v>
+        <v>73.05417704582214</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -1434,25 +1434,25 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1.716034650802612</v>
+        <v>57.43383383750916</v>
       </c>
       <c r="B39" t="n">
-        <v>1509.4296875</v>
+        <v>42.515625</v>
       </c>
       <c r="C39" t="n">
-        <v>6.9</v>
+        <v>3.8</v>
       </c>
       <c r="D39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>0.453843355178833</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0.4555583000183105</v>
+        <v>57.43382906913757</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -1460,13 +1460,13 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>10.85743951797485</v>
+        <v>95.51131868362427</v>
       </c>
       <c r="B40" t="n">
-        <v>1509.8046875</v>
+        <v>31.375</v>
       </c>
       <c r="C40" t="n">
-        <v>11.3</v>
+        <v>9</v>
       </c>
       <c r="D40" t="n">
         <v>4</v>
@@ -1475,10 +1475,10 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0.3169059753417969</v>
+        <v>2.995203733444214</v>
       </c>
       <c r="G40" t="n">
-        <v>0.3184688091278076</v>
+        <v>43.28196573257446</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -1486,13 +1486,13 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>3.430304288864136</v>
+        <v>80.5112829208374</v>
       </c>
       <c r="B41" t="n">
-        <v>1509.80859375</v>
+        <v>27.6875</v>
       </c>
       <c r="C41" t="n">
-        <v>5.3</v>
+        <v>15.5</v>
       </c>
       <c r="D41" t="n">
         <v>4</v>
@@ -1501,10 +1501,10 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>1.552063941955566</v>
+        <v>3.091278076171875</v>
       </c>
       <c r="G41" t="n">
-        <v>1.553599834442139</v>
+        <v>37.34941697120667</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -1512,13 +1512,13 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>7.940751791000366</v>
+        <v>94.10230398178101</v>
       </c>
       <c r="B42" t="n">
-        <v>1509.80859375</v>
+        <v>38.78125</v>
       </c>
       <c r="C42" t="n">
-        <v>12.1</v>
+        <v>15.4</v>
       </c>
       <c r="D42" t="n">
         <v>4</v>
@@ -1527,10 +1527,10 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0.3915088176727295</v>
+        <v>2.612574815750122</v>
       </c>
       <c r="G42" t="n">
-        <v>0.3939275741577148</v>
+        <v>40.97972989082336</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -1538,25 +1538,25 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>12.52107214927673</v>
+        <v>121.0973088741302</v>
       </c>
       <c r="B43" t="n">
-        <v>1509.984375</v>
+        <v>34.78125</v>
       </c>
       <c r="C43" t="n">
-        <v>10</v>
+        <v>7.4</v>
       </c>
       <c r="D43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>1.446927785873413</v>
+        <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>1.448587656021118</v>
+        <v>121.0972499847412</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -1564,13 +1564,13 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>10.58960342407227</v>
+        <v>149.4924519062042</v>
       </c>
       <c r="B44" t="n">
-        <v>1510.25390625</v>
+        <v>40.09375</v>
       </c>
       <c r="C44" t="n">
-        <v>8.199999999999999</v>
+        <v>5</v>
       </c>
       <c r="D44" t="n">
         <v>4</v>
@@ -1579,10 +1579,10 @@
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>1.522054433822632</v>
+        <v>3.727458000183105</v>
       </c>
       <c r="G44" t="n">
-        <v>1.523772478103638</v>
+        <v>52.33642387390137</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -1590,25 +1590,25 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>11.24179005622864</v>
+        <v>109.82266497612</v>
       </c>
       <c r="B45" t="n">
-        <v>1510.83203125</v>
+        <v>35.140625</v>
       </c>
       <c r="C45" t="n">
-        <v>10.2</v>
+        <v>4.4</v>
       </c>
       <c r="D45" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>1.56652569770813</v>
+        <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>1.568768978118896</v>
+        <v>109.8225989341736</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -1616,25 +1616,25 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>4.401284456253052</v>
+        <v>100.7978947162628</v>
       </c>
       <c r="B46" t="n">
-        <v>1510.83203125</v>
+        <v>35.21875</v>
       </c>
       <c r="C46" t="n">
-        <v>11.3</v>
+        <v>5.1</v>
       </c>
       <c r="D46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>1.489950180053711</v>
+        <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>1.492054462432861</v>
+        <v>100.7978558540344</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -1642,25 +1642,25 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>9.897516250610352</v>
+        <v>87.02002286911011</v>
       </c>
       <c r="B47" t="n">
-        <v>1510.89453125</v>
+        <v>44.96875</v>
       </c>
       <c r="C47" t="n">
-        <v>9.1</v>
+        <v>3.9</v>
       </c>
       <c r="D47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>0.3515493869781494</v>
+        <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>0.3532202243804932</v>
+        <v>87.02001690864563</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -1668,25 +1668,25 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>9.118991136550903</v>
+        <v>67.3652331829071</v>
       </c>
       <c r="B48" t="n">
-        <v>1510.89453125</v>
+        <v>40.03125</v>
       </c>
       <c r="C48" t="n">
-        <v>10.6</v>
+        <v>3.7</v>
       </c>
       <c r="D48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>1.50508451461792</v>
+        <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>1.506625652313232</v>
+        <v>67.36517119407654</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -1694,25 +1694,25 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>13.59402275085449</v>
+        <v>40.94291424751282</v>
       </c>
       <c r="B49" t="n">
-        <v>1510.89453125</v>
+        <v>34.40625</v>
       </c>
       <c r="C49" t="n">
-        <v>10.1</v>
+        <v>4.4</v>
       </c>
       <c r="D49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>1.445708274841309</v>
+        <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>1.447296619415283</v>
+        <v>40.94286298751831</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -1720,25 +1720,25 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>9.183413505554199</v>
+        <v>68.04189300537109</v>
       </c>
       <c r="B50" t="n">
-        <v>1511.1328125</v>
+        <v>19.734375</v>
       </c>
       <c r="C50" t="n">
-        <v>10.8</v>
+        <v>10</v>
       </c>
       <c r="D50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>1.43329644203186</v>
+        <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>1.434942245483398</v>
+        <v>68.04185700416565</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
@@ -1746,13 +1746,13 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>13.14925694465637</v>
+        <v>149.0001132488251</v>
       </c>
       <c r="B51" t="n">
-        <v>1511.46484375</v>
+        <v>19.5</v>
       </c>
       <c r="C51" t="n">
-        <v>10</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D51" t="n">
         <v>4</v>
@@ -1761,10 +1761,10 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>1.531296491622925</v>
+        <v>3.00985312461853</v>
       </c>
       <c r="G51" t="n">
-        <v>1.532980442047119</v>
+        <v>60.81364107131958</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
@@ -1772,25 +1772,25 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>11.57462024688721</v>
+        <v>116.0841212272644</v>
       </c>
       <c r="B52" t="n">
-        <v>1511.46484375</v>
+        <v>21.875</v>
       </c>
       <c r="C52" t="n">
-        <v>10.3</v>
+        <v>5</v>
       </c>
       <c r="D52" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>1.464968919754028</v>
+        <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>1.466602563858032</v>
+        <v>116.0840501785278</v>
       </c>
       <c r="H52" t="n">
         <v>0</v>
@@ -1798,25 +1798,25 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>11.58727788925171</v>
+        <v>109.3119170665741</v>
       </c>
       <c r="B53" t="n">
-        <v>1511.93359375</v>
+        <v>20.421875</v>
       </c>
       <c r="C53" t="n">
-        <v>9.300000000000001</v>
+        <v>4.7</v>
       </c>
       <c r="D53" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>1.522054672241211</v>
+        <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>1.523861885070801</v>
+        <v>109.3118767738342</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
@@ -1824,25 +1824,25 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>11.22345447540283</v>
+        <v>229.9391770362854</v>
       </c>
       <c r="B54" t="n">
-        <v>1511.9375</v>
+        <v>20.8125</v>
       </c>
       <c r="C54" t="n">
-        <v>8.800000000000001</v>
+        <v>4.5</v>
       </c>
       <c r="D54" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>1.452330112457275</v>
+        <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>1.454082727432251</v>
+        <v>229.9391229152679</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
@@ -1850,25 +1850,25 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>3.621444463729858</v>
+        <v>71.94218492507935</v>
       </c>
       <c r="B55" t="n">
-        <v>1511.94140625</v>
+        <v>20.484375</v>
       </c>
       <c r="C55" t="n">
-        <v>13.1</v>
+        <v>5.7</v>
       </c>
       <c r="D55" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E55" t="n">
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>1.520708799362183</v>
+        <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>1.522382974624634</v>
+        <v>71.94211673736572</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -1876,13 +1876,13 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>12.05659079551697</v>
+        <v>171.5674619674683</v>
       </c>
       <c r="B56" t="n">
-        <v>1511.94921875</v>
+        <v>20.859375</v>
       </c>
       <c r="C56" t="n">
-        <v>10.7</v>
+        <v>7.3</v>
       </c>
       <c r="D56" t="n">
         <v>4</v>
@@ -1891,10 +1891,10 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>0.3717708587646484</v>
+        <v>3.290996074676514</v>
       </c>
       <c r="G56" t="n">
-        <v>0.3734982013702393</v>
+        <v>81.51416897773743</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
@@ -1902,25 +1902,25 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>10.68418478965759</v>
+        <v>93.42482709884644</v>
       </c>
       <c r="B57" t="n">
-        <v>1514.32421875</v>
+        <v>20.734375</v>
       </c>
       <c r="C57" t="n">
-        <v>8.199999999999999</v>
+        <v>6.5</v>
       </c>
       <c r="D57" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E57" t="n">
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>1.628901481628418</v>
+        <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>1.630803346633911</v>
+        <v>93.42480516433716</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -1928,13 +1928,13 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>10.82381558418274</v>
+        <v>204.0498929023743</v>
       </c>
       <c r="B58" t="n">
-        <v>1514.32421875</v>
+        <v>19.9375</v>
       </c>
       <c r="C58" t="n">
-        <v>10.1</v>
+        <v>8.9</v>
       </c>
       <c r="D58" t="n">
         <v>4</v>
@@ -1943,10 +1943,10 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>1.628249645233154</v>
+        <v>3.308865070343018</v>
       </c>
       <c r="G58" t="n">
-        <v>1.630011796951294</v>
+        <v>107.5027179718018</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -1954,25 +1954,25 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>10.40878295898438</v>
+        <v>95.01514601707458</v>
       </c>
       <c r="B59" t="n">
-        <v>1514.32421875</v>
+        <v>20.8125</v>
       </c>
       <c r="C59" t="n">
-        <v>10.4</v>
+        <v>13.3</v>
       </c>
       <c r="D59" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E59" t="n">
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>1.457972526550293</v>
+        <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>1.460432767868042</v>
+        <v>95.01511788368225</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
@@ -1980,25 +1980,25 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>14.37377834320068</v>
+        <v>109.1969590187073</v>
       </c>
       <c r="B60" t="n">
-        <v>1514.32421875</v>
+        <v>19.859375</v>
       </c>
       <c r="C60" t="n">
-        <v>10</v>
+        <v>6.5</v>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E60" t="n">
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>1.486737489700317</v>
+        <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>1.48843240737915</v>
+        <v>109.1969089508057</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
@@ -2006,25 +2006,25 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>10.56781244277954</v>
+        <v>105.5565929412842</v>
       </c>
       <c r="B61" t="n">
-        <v>1514.32421875</v>
+        <v>20.671875</v>
       </c>
       <c r="C61" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>1.48133373260498</v>
+        <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>1.482977867126465</v>
+        <v>105.5565619468689</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
@@ -2032,25 +2032,25 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>3.619588851928711</v>
+        <v>31.90827894210815</v>
       </c>
       <c r="B62" t="n">
-        <v>1514.32421875</v>
+        <v>26.796875</v>
       </c>
       <c r="C62" t="n">
-        <v>5.6</v>
+        <v>7.9</v>
       </c>
       <c r="D62" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>1.437713384628296</v>
+        <v>0</v>
       </c>
       <c r="G62" t="n">
-        <v>1.439305305480957</v>
+        <v>31.90825986862183</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
@@ -2058,25 +2058,25 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>8.809430599212646</v>
+        <v>52.95605301856995</v>
       </c>
       <c r="B63" t="n">
-        <v>1514.32421875</v>
+        <v>21.828125</v>
       </c>
       <c r="C63" t="n">
-        <v>11.8</v>
+        <v>5.3</v>
       </c>
       <c r="D63" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>0.3265001773834229</v>
+        <v>0</v>
       </c>
       <c r="G63" t="n">
-        <v>0.3280789852142334</v>
+        <v>52.95597910881042</v>
       </c>
       <c r="H63" t="n">
         <v>0</v>
@@ -2084,13 +2084,13 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>9.809545755386353</v>
+        <v>94.91445803642273</v>
       </c>
       <c r="B64" t="n">
-        <v>1514.32421875</v>
+        <v>20.421875</v>
       </c>
       <c r="C64" t="n">
-        <v>10.4</v>
+        <v>5.5</v>
       </c>
       <c r="D64" t="n">
         <v>4</v>
@@ -2099,10 +2099,10 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>1.435290098190308</v>
+        <v>3.651123762130737</v>
       </c>
       <c r="G64" t="n">
-        <v>1.436878681182861</v>
+        <v>44.7390661239624</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -2110,25 +2110,25 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>6.040205478668213</v>
+        <v>49.85166525840759</v>
       </c>
       <c r="B65" t="n">
-        <v>1514.32421875</v>
+        <v>19.84375</v>
       </c>
       <c r="C65" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="D65" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E65" t="n">
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>1.502256631851196</v>
+        <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>1.50404691696167</v>
+        <v>49.85157608985901</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -2136,25 +2136,25 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>9.838013410568237</v>
+        <v>40.76638102531433</v>
       </c>
       <c r="B66" t="n">
-        <v>1514.32421875</v>
+        <v>21.796875</v>
       </c>
       <c r="C66" t="n">
-        <v>11.4</v>
+        <v>4.6</v>
       </c>
       <c r="D66" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>0.3295505046844482</v>
+        <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>0.3311994075775146</v>
+        <v>40.76634287834167</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -2162,25 +2162,25 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>9.913764476776123</v>
+        <v>43.52314376831055</v>
       </c>
       <c r="B67" t="n">
-        <v>1514.32421875</v>
+        <v>20.96875</v>
       </c>
       <c r="C67" t="n">
-        <v>10</v>
+        <v>5.8</v>
       </c>
       <c r="D67" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>1.479658842086792</v>
+        <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>1.482023239135742</v>
+        <v>43.52306485176086</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -2188,25 +2188,25 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>4.961272954940796</v>
+        <v>57.20432019233704</v>
       </c>
       <c r="B68" t="n">
-        <v>1514.99609375</v>
+        <v>21.390625</v>
       </c>
       <c r="C68" t="n">
-        <v>7.6</v>
+        <v>4.7</v>
       </c>
       <c r="D68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E68" t="n">
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>1.512712478637695</v>
+        <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>1.514587163925171</v>
+        <v>57.20421242713928</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>

</xml_diff>